<commit_message>
Changed documents to match new code
</commit_message>
<xml_diff>
--- a/API-Design.xlsx
+++ b/API-Design.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Design" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="API Design" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Design'!$A$1:$K$22</definedName>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1779,7 +1779,7 @@
         <is>
           <t>Path param: id
 JSON body:
-status (PENDING/SHIPPED)</t>
+status (PENDING/CONFIRMED/PROCESSING/SHIPPED/DELIVERED/CANCELLED/REFUNDED)</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1788,6 +1788,64 @@
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ECOM-002h</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Verify email address</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Verify Email</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>[GET] /api/users/verify-email</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Client (Web/Mobile)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>User Service</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>N/A (public)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Query param:
+token</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>id, username, email, firstName, lastName, roles</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t>Update</t>
         </is>

</xml_diff>